<commit_message>
Add CA leads Delhi NCR - 2026-04-06 10:59
</commit_message>
<xml_diff>
--- a/CA_20260406_1046.xlsx
+++ b/CA_20260406_1046.xlsx
@@ -1474,7 +1474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1538,6 +1538,3576 @@
       <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Fetched At</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>L Singh &amp; Associates Chartered Accountants - Company and GST Registration, Income Tax Return Filing and Best CA Firm</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>+91 99994 79431</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>http://www.calsingh.com/</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>B-18 Basement, Community Centre, B1 Market, Pocket B 1, Super Bazar, Janakpuri, New Delhi, Delhi, 110058, India</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>CA In Delhi</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>+91 99114 92897</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>https://caindelhi.in/</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="n"/>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>CA Naresh Kansal</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>+91 98731 92124</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>https://canareshkansal.com/</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Office No. 346, 3rd Floor Vardhman Premium Mall, Near Tarun Enclave Opposite kali mata mandir, sector 3 rohini, Outer Ring Rd, Deepali, Pitampura, Delhi, 110034, India</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>CA Gajanand Baheti &amp; Co., Chartered Accountants (CA Near Me)</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>+91 78219 23970</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>https://wa.me/917821923970?text=Hello%20CA%20Gajanand</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Second Floor, 57, Mausam Vihar, Delhi, 110051, India</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>AMM &amp; Associates Chartered Accountants</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>+91 93128 37129</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>http://www.certifiedcorporateaccountant.com/</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>A-100, Bipin Chandra Pal Marg, Block A, Chittaranjan Park, New Delhi, Delhi 110019, India</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Sanjay Tyagi &amp; Associates, Best CA Firm, Best NGO consultant</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>+91 99994 22224</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>H-30C, near Aruna Park, Shakarpur, New Delhi, Delhi 110092, India</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>CA HARPREET SABHARWAL &amp; ASSOCIATES ( CHARTERED ACCOUNTANTS)</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>+91 99588 38456</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr"/>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Income tax help association</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>FLUID GYM, C- Opposite, 75, Gurudwara Rd, C block, Nanak Pura, Hari Nagar, New Delhi, Delhi, 110064, India</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Chartered accountants in Karol Bagh</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>+91 99909 99281</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>http://myca.live/</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Certified public accountant</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>2029, Bank St, near Shreem Jewellers, Block 47, Beadonpura, Karol Bagh, New Delhi, Delhi, 110005, India</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Rajput Jain &amp; Associates</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>+91 98113 22785</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>http://www.carajput.com/</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Tax consultant</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>P 6/90, Connaught Circus Near Palika Bazar, Revoli Cinema, Connaught Place, New Delhi, Delhi 110001, India</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Harsh Gupta &amp; Associates (Chartered Accountant Firm)</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>+91 91367 10504</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>https://charteredpride.in/</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>First Floor, Metro Station Krishna Nagar, F-7/31, Pink Line, near Gupta Opticals, Block F, Krishna Nagar, New Delhi, Delhi, 110051, India</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>AMBK &amp; ASSOCIATES | Chartered Accountant Firm in Delhi</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>+91 99991 82203</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>https://ambkandassociates.com/</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>2206/2, 1st Floor, Chah indara, Bhagirath Palace, Chhippy Wada, Chandni Chowk, New Delhi, Delhi, 110006, India</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>CA RAJENDER ARORA</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>+91 98911 12120</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Certified public accountant</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>4th Floor, DSM 401, DLF TOWERS, 15, Shivaji Marg, Moti Nagar, House Complex Market, Karampura Industrial Area, Zakhira, New Delhi, Delhi, 110015, India</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Ca Atul Mangal &amp; Co</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>+91 92120 07566</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>http://www.camangal.com/</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>19, Flat, Block A, A St, opp. Ardee Montessori House, DDA Flats, Munirka, New Delhi, Delhi 110067, India</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Malik Girish Anand &amp; Co.| Accounting Services | Corporate Tax| CA Firm in Delhi |GST Return | Income Tax Return | ITR Filing</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>+91 98100 46556</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>https://camalikgirishanand.co.in/</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>FF-101, SARINE SONIA SADAN COMMUNITY CENTRE VIKAS PURI, NEW DELHI, NEAR PVR VIKAS PURI, New Delhi, Delhi 110018, India</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Manish Anil Gupta And Co</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>+91 99994 55360</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.manishanilgupta.com/</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Certified public accountant</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>4/1 Springhouse, Prem Nagar, Janakpuri, New Delhi, Delhi 110058, India</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Agarwal Taxcon Private Limited</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>+91 75036 38500</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>https://agarwaltaxcon.in/</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Accountant</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Khosla Complex, B-10, Gagan Vihar Extension, Gagan Vihar, Krishna Nagar, Delhi, 110092, India</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>D D Agrawal &amp; Co. Chartered Accountants</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>+91 95821 01001</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>http://dda-co.com/</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Certified public accountant</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>413 &amp; 814A, Vikasdeep Building Laxmi Nagar District Centre, Swasthya Vihar, New Delhi, Delhi 110092, India</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>V Sahai Tripathi &amp; Co</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>+91 99995 61115</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>http://www.sahaitripathi.com/</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>8E, Hansalaya 15, Barakhamba Rd, Connaught Place, New Delhi, Delhi 110001, India</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>SDM &amp; CO ( CA MD SABIR ALI), Chartered Accountants</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>+91 99716 16576</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>http://casdm.in/</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>2nd Floor, Surya Plaza Building, K-185/2, above SBI Bank, Block D, Okhla, New Delhi, Delhi 110025, India</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>C P Agrawal &amp; Associates - CA in Delhi</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>+91 93112 21571</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cacpa.in/</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Ground Floor, 142, Chitra Vihar, Swasthya Vihar, Delhi, 110092, India</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>CA Nitender Arya | Best CA firm in South Delhi</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>+91 70153 48484</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr"/>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>OFFICE NO C, 49, near DIVINE GYM, Rajpur Khurd Extension, Chhatarpur, Delhi, New Delhi, Delhi 110068, India</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>S Daryani &amp; Associates</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>+91 98114 28949</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>http://www.sushildaryani.com/</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Golf View Apartments, A-60, Press Enclave Marg, Saket, New Delhi, Delhi 110017, India</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Ca in Delhi - CA M C Maheshwari &amp; Company - Ca firm - Chartered Accountant Delhi</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>+91 98993 50801</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Building No.17, 1st Floor, Yusuf Sarai Main Road, Near Green Park Metro Station, New Delhi, Delhi 110016, India</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Sunil Arora &amp; Associates - Best Chartered Accountants firm in South Delhi India</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>+91 11 4175 9993</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>http://www.casunilarora.com/</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>A-1/118, Block A 1, Nauroji Nagar, Safdarjung Enclave, New Delhi, Delhi 110029, India</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Nitin Mittal &amp; Co.</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>+91 98101 47514</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>http://nmcindia.net/</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>C 21b, South Extension I, Block C, New Delhi, Delhi 110049, India</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>SARIKA &amp; CO., Chartered Accountants</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>+91 99104 72202</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>http://www.sarikaca.com/</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Certified public accountant</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>6155/1, Santushti Apartments, D6, Sector D, Vasant Kunj, New Delhi, Delhi 110070, India</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>K.B. Chandna and Co.</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>+91 98110 73984</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kbcca.com/</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>E-27, South Extension II, Block C, New Delhi, Delhi 110049, India</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>MNRS &amp; Associates, Chartered Accountant (CA) Firm In Delhi. Tax, Audit and FEMA Consultants in Delhi/NCR</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>+91 98109 02950</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>http://mnrsindia.com/</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>1st &amp;, 2nd Floor, I-35B, I Block Rd, Central Market, Lajpat Nagar II, Lajpat Nagar, New Delhi, Delhi 110024, India</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Mayank Khatri &amp; Company Chartered Accountants</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>+91 98993 92710</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Certified public accountant</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Block H 6, Malviya Nagar, New Delhi, Delhi 110017, India</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Srivastava Kumar &amp; Co. Chartered Accountants</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>+91 98110 73788</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>https://www.skcca.com/</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>404, 4th floor, Block G 6, Nehru Place, New Delhi, Delhi 110019, India</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Manchanda and Associates | Chartered Accountants &amp; ITR Experts</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>+91 93183 36610</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr"/>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Shop no-6, First Floor, Block-B, DDA Flats, Janta Market, Kalkaji, New Delhi, Delhi 110019, India</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>PKG Consultancy-CA Firm in Kalkaji|LLP|NGO|GST|Company Registration|ITR</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>+91 83779 81363</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>http://www.pkgconsultancy.com/</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Certified public accountant</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>J1/150, Ground Floor, near kwality Sweets &amp; Restaurant, DDA Flats Kalkaji, New Delhi, Delhi 110019, India</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>M/s. Shiwali &amp; Co. Chartered Accountants</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>+91 92660 32777</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>http://www.cashiwali.com/</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>412, opposite Punjab National Bank, Durga Vihar, Devli, branch, New Delhi, Delhi, 110062, India</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>PUNEET SHIKHA GUPTA &amp; ASSOCIATES</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>+91 98187 47300</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>http://www.psga.in/</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>C 6 GF, Metro Station-Saket, near, Malviya Nagar Rd, Block C, Geetanjali Enclave, Malviya Nagar, New Delhi, Delhi 110017, India</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J35" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Kishore Gupta &amp; Co. - Chartered Accountants | Connaught Place | Tax Audit | Company Registration | GST Registration | ITR</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>+91 97110 33545</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>http://kgcoca.com/</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Flat No.11, C-41, Block C, Connaught Place, New Delhi, Delhi 110001, India</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>G K Kedia &amp; Co., Connaught Place Office</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>+91 11 4625 9900</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>https://www.gkkediaandco.com/</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>812, Naurang House, 21, KG Marg, Atul Grove Road, Janpath, Connaught Place, New Delhi, Delhi 110001, India</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="I37" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>T R Chadha &amp; Co.</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>+91 11 4325 9900</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>http://www.trchadha.com/</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Block B,B, 30, Connaught Cir, Block H, Connaught Place, New Delhi, Delhi 110001, India</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>R Arora &amp; Associates</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>+91 11 2335 0617</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>http://www.r-arora.com/</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>612 Surya Kiran, 19 Kasturba Gandhi Marg, Connaught Place, Delhi, 110001, India</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>B R Maheswari &amp; Co LLP</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>+91 11 4340 2222</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>http://www.brmco.com/</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>M-118, Block M, Connaught Place, New Delhi, Delhi 110001, India</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>Manoj Pahwa And Associate</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>+91 11 4702 6276</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>https://manoj-pahwa.grexa.site/</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>BMC House, N Block, 305, Middle Cir, Block N, Connaught Place, New Delhi, Delhi 110001, India</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>J S SHARMA AND CO</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>+91 98100 29426</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>http://jssandco.in/</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Certified public accountant</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>1605 NIRMAL TOWER, 26, Barakhamba Rd, Connaught Place, New Delhi, Delhi 110001, India</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>AAGS &amp; Co.</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>+91 11 4308 0505</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>http://www.eindiacharteredaccountants.com/</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>9C 9th Floor, Atma Ram House, 1, Tolstoy Rd, Connaught Place, New Delhi, Delhi 110001, India</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Deepak Gulati &amp; Associates</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>+91 98100 06345</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>http://www.dga.in/</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>23, Hanuman Rd, Hanuman Road Area, Connaught Place, New Delhi, Delhi 110001, India</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>VICKY KAPOOR &amp; ASSOCIATES</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>+91 98107 60659</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>http://cavka.in/</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>Accounting firm</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>Indra Prakash Building, 1109, 11th Floor, Barakhamba Rd, New Delhi, Delhi 110001, India</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Dinesh Aarjav and Associates Chartered Accountants (Branch Office)</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>+91 11 4309 5042</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>http://www.dineshaarjav.com/</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Accounting firm</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>411, Kailash Building, 26, KG Marg, Connaught Place, Delhi, New Delhi, Delhi 110001, India</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>S. Ramanand Aiyar &amp; Co.</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>+91 11 2331 9284</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>http://www.sraco.in/</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>19, KG Marg, Atul Grove Road, Janpath, Connaught Place, New Delhi, Delhi 110001, India</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I47" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J47" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>V K Verma &amp; Company</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>+91 11 2341 5811</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>http://www.vkvermaco.com/</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>C-37, Block C, Connaught Place, New Delhi, Delhi 110001, India</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>P.N. Khanna &amp; Co</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>+91 11 4940 8253</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr"/>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>806, Barakhamba Rd, Barakhamba, New Delhi, Delhi 110001, India</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I49" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J49" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>P N A M &amp; Co. LLP</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>+91 11 2140 0294</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>https://pnam.co/</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>F-14/15 2nd Floor, Shivam House, 14, Middle Cir, Block F, Connaught Place, New Delhi, Delhi 110001, India</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>Arpit Suri &amp; Co. - Best CA Firm In West Delhi</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>+91 98730 17270</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>https://www.arpitsuriandco.com/</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>Certified public accountant</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>C-3/ 324A, Block C3A, Block C3, Janakpuri, New Delhi, Delhi, 110058, India</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H51" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I51" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J51" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>Aakash Garg &amp; Co Chartered Accountants, CA Firm in Delhi, CA in Delhi</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>+91 88103 61282</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>http://www.agargca.com/</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Certified public accountant</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>WZ-9A, Vishnu Park, near Post office, Chand Nagar, New Delhi, Delhi 110018, India</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>MUKESH DUTT AND ASSOCIATES- CA Firm in Uttam Nagar/Janakpuri West Delhi for GST, TAX etc.</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>+91 84488 60689</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr"/>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>Certified public accountant</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>near Laal Mandir, Indra Park Extension, Block A, Ram Datt Enclave, Uttam Nagar, New Delhi, Delhi, 110059, India</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="I53" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J53" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Ankit Sehra &amp; Associates |Income Tax Return| Company and GST Registration| Best CA Firm In Delhi</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>+91 98915 71973</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>http://ankitsehra.com/</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Certified public accountant</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>3rd Floor, Westend Mall, Unit No - 304, near by Janakpuri West Metro Station, Janakpuri District Center, Janakpuri, New Delhi, Delhi, 110058, India</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>Gst Registration In Delhi | Income Tax Return | Company Audit | Company Registration | Ambience India Ca Firm In Delhi</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>+91 81785 55520</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>https://aiadvisory.in/</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>B120, 2nd Floor, near Metro Pillar No- 547, Ganesh Nagar, New Delhi, Delhi 110018, India</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H55" s="3" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="I55" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J55" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Vishal Madan &amp; Co | GST Registration, Business Tax Filing , Personal Tax Filing</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>+91 92122 09250</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>https://vishalmadanca.com/</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>25/6, Chhoti Subji Mandi, Janakpuri, New Delhi, Delhi, 110058, India</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>Naresh K Bhatia &amp; Associates | ITR | Chartered Accountant | CA in Delhi | CA in West Delhi | CA in Uttam Nagar | Filling</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>+91 70099 39796</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr"/>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>1st Floor, wZ 66A, Dayal Sar Road, South Extension 1, Block K, Param Puri, Uttam Nagar, New Delhi, Delhi, 110059, India</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I57" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J57" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Sawhney &amp; Sawhney Chartered Accountants</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>+91 83770 76697</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>http://snsindia.in/</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>First Floor, DDA Market, F5, Block, near St. Mary's school, Ambica Vihar, Paschim Vihar, Delhi, 110087, India</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>NHRG &amp; Associates (CA) (GST Expert)</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>+91 90688 33883</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>http://www.nhrg.in/</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>Certified public accountant</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>First Floor, A-3/8, opposite Bank of Baroda, Paschim Vihar, Delhi, 110063, India</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G59" s="3" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H59" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I59" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J59" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Maini Singh &amp; Co.</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>+91 96677 60697</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>http://www.mainisingh.in/</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>Certified public accountant</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>A82, A Block, Vishal Enclave, Tagore Garden Extension, New Delhi, Delhi, 110027, India</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>Vaaridhi Consulting Co - CA in Dwarka, Delhi | CA Firm in West Delhi - GST Consultant/Tax Consultant/ITR Filling etc.</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>+91 97117 49053</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr"/>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>622, Uttam Vihar, Block B, DDA FLATS, Bindapur, New Delhi, Delhi, 110059, India</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G61" s="3" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H61" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="I61" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J61" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>CA. Saroj Kumar Jha/CA in Uttam Nagar/Chartered Accountant</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>+91 97488 73205</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr"/>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>Certified public accountant</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>E-227A, E Block, Mansa Ram Park, Uttam Nagar, New Delhi, Delhi, 110059, India</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>Pradeep JB and Associates CA Firm|GST Return| ITR Return |Income Tax| Pashim Vihar |Delhi</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>+91 95994 97968</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr"/>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t>487/49, National Market, near Bhatnagar International School, Peera Garhi, Paschim Vihar, Delhi, 110087, India</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G63" s="3" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H63" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I63" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J63" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>R S KAPOOR &amp; CO. ( C.A. , Advocate ) - Best CA Firm in Delhi - GST Consultant,GST Registration,Income Tax, Auditing</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>+91 98718 18553</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr"/>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>G.K. House, 1139, Mukherjee Nagar, Delhi, 110033, India</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>CA in Delhi || ADY &amp; Co. Chartered Accountant</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>+91 99998 13738</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>https://caindelhi.org/</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
+          <t>A 28 2nd Floor Above Canara Bank Ramgarh, Ramgarh Village, Jahangirpuri GT Karnal Road, Metro Piller no 151, near Jahangirpuri Metro Station, Delhi, 110033, India</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H65" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I65" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J65" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>Adlakha Kukreja and Co - CA Firm</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>+91 98998 22054</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>https://akcoindia.com/</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>2nd Foor, Q-7, Model Town Phase I, Mukherjee Nagar, Delhi, 110009, India</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>CA B K Goyal &amp; Co LLP Chartered Accountants - Best CA in Delhi</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>+91 99717 82649</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cabkgoyal.com/ca-in-delhi/</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="n"/>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H67" s="3" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="I67" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J67" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>Goyal K and Associates CA |Accounting | GST |Company | Registeration |CA Firm in Delhi | ITR Filling |Rohini |Pitampura</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>+91 98137 63364</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>http://www.goyalk.com/</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>B-6/178 FF, near Swimming Pool, C Block, Sector 8B, Sector 8, Rohini, New Delhi, Delhi, 110085, India</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t>Mangla &amp; Associates, CA, Pitampura, Delhi</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>+91 99991 81231</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr"/>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t>RU-404, Outer Ring Rd, Block RU, Uttari Pitampura, Pitampura, Delhi, 110034, India</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G69" s="3" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H69" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I69" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J69" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>Goyal Mittal And Co</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>+91 97803 83400</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr"/>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>305, ADARSH COMPLEX, Wazirpur Industrial Area, Ashok Vihar, New Delhi, Delhi, 110052, India</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>V D JAIN &amp; CO. - CA in Rohini, GST Income Tax MCA compliances ,Company/Firm Registration, MSME, Trademark ,Auditing</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>+91 85270 48978</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>https://vdjc.co.in/</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t>SG shopping mall tower, 308, DC Chowk, Rajapur, Sector 9, Rohini, Delhi, 110085, India</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G71" s="3" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H71" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I71" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J71" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>MAURYA &amp; CO (CA &amp; Advocate)</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>+91 97160 61648</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr"/>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>Certified public accountant</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>L-158, Grnd floor KH 1280, Gali No 15, Bhatta Rd, Swaroop Nagar, Delhi, 110042, India</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>Madhu Sudan &amp; Co - Chartered Accountant in North Delhi</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>+91 98112 52448</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr"/>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>Certified public accountant</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="inlineStr">
+        <is>
+          <t>F-14/57, 11nd Floor, Model Town Phase 2, Delhi, 110033, India</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G73" s="3" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H73" s="3" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="I73" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J73" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>CA Durgesh Tripathi, Chartered accountant</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>+91 97161 53750</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/ca-durgesh-tripathi-717002203?utm_source=share&amp;utm_campaign=share_via&amp;utm_content=profile&amp;utm_medium=android_app</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>Chartered accountant</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>A-511/1, Nathu Pura, Nathupura, Burari, Delhi, 110084, India</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>Chartered Accountant (CA)</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps via Apify</t>
+        </is>
+      </c>
+      <c r="J74" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06 10:59</t>
         </is>
       </c>
     </row>

</xml_diff>